<commit_message>
Testcase and Test log done
</commit_message>
<xml_diff>
--- a/Source/docs/testCases/UserRoles-defect-log.xlsx
+++ b/Source/docs/testCases/UserRoles-defect-log.xlsx
@@ -1,23 +1,20 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Defect Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Methodology &amp; Notes" sheetId="2" state="visible" r:id="rId2"/>
-  </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Log'!$A$4:$I$10</definedName>
-  </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>openpyxl</dc:creator>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-09-17T13:01:48Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-09-17T13:01:48Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="7">
@@ -236,7 +233,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -519,13 +516,31 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Defect Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Methodology &amp; Notes" sheetId="2" state="visible" r:id="rId2"/>
+  </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Log'!$A$4:$I$11</definedName>
+  </definedNames>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -549,7 +564,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Code-inspection based — not confirmed via test execution. Source: Source/docs/testCases/UserRoles-defect-log.md</t>
+          <t>Code-inspection based — not confirmed via test execution. Source: Source/docs/testCases/UserRoles-defect-log.md. Re-verified 2026-09-18 against current source (DEF-001..005 and NOTE-001 unchanged; DEF-006 added).</t>
         </is>
       </c>
     </row>
@@ -882,8 +897,55 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="105" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>DEF-UserRoles-006</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>GetUserRoleById returns an empty 204 for an unknown RoleId while the three mutating endpoints return 404 with a message for the same condition</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Open — pending runtime confirmation</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>TC-UserRoles-020, TC-UserRoles-024, TC-UserRoles-030</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>UserRolesService.cs, GetUserRoleByIdAsync (data == null branch sets StatusCode = ErrorCodes.NoRecordFound = 204) vs. SaveUserRoleAsync/UpdateUserRoleStatusAsync/DeleteUserRoleAsync (unknown-RoleId branch sets StatusCode = ErrorCodes.NotFound = 404, StatusMessage = ErrorMessages.RoleNotFound); BaseController.GetResponseByStatusCode: Status204NoContent =&gt; NoContent() (discards resultArgs entirely - true empty body) vs. Status404NotFound =&gt; NotFound(resultArgs) (JSON body with statusMessage "This role no longer exists.").</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Fetching a role by an id that doesn't exist should surface the same class of error the other three UserRoles endpoints use for the identical condition, so a caller/frontend can distinguish "this id does not exist" from "the request succeeded with nothing to show."</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>GET GetUserRoleById?roleId=&lt;unknown&gt; returns HTTP 204 No Content with a completely empty response body (no statusCode/statusMessage/resultData at all). A frontend that treats any non-error HTTP status as success would render a blank edit form with no error message instead of a "role not found" message.</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Change GetUserRoleByIdAsync's not-found branch to ErrorCodes.NotFound/ErrorMessages.RoleNotFound, matching the other three UserRoles endpoints, unless product intentionally wants a bare empty response here - confirm with the business owner before changing shared 204 handling elsewhere in the codebase.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I10"/>
+  <autoFilter ref="A4:I11"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -892,13 +954,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -946,6 +1008,20 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Re-verification pass — 2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="75" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>This environment still cannot run the NUnit suite or the Selenium/BDD suite (same blockers as above), so this pass re-read UserRolesController.cs, UserRolesService.cs, UserRolesRepository.cs, 004_Acutis_UserRoles.sql, UserRolesInput.cs/UserRoleStatusInput.cs/UserRolesOutput.cs, UserRolesValidator.ts, UserRolesApiNegativeTests.cs, DisablePolicy.cs, BaseController.cs, and MessageCatalog.cs end-to-end. DEF-UserRoles-001 through 005 and NOTE-001 all still match the current source exactly (no code changes to this module since the prior pass). One new defect, DEF-UserRoles-006, was found by tracing GetUserRoleById's not-found branch against BaseController's status-code-to-HTTP-response mapping, which the prior pass had not done.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>